<commit_message>
Update analysis and educational plan files across multiple programs
- Modified various Excel files related to grading reporting, grading scales, Bloom's taxonomy, examination forms, and consistency in phrasing for the following programs: IIT, IHV, IKS, and ISLL.
- Updated markdown files for educational plans, changing program codes and course references to reflect the latest curriculum changes.
- Corrected links and course names in markdown files to ensure accuracy and consistency.
- Adjusted the number of findings in the analysis reports to match the updated data.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DBIMA</t>
+          <t>DITMG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,24 +482,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bullet beskriver val mellan flera kurser</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`Datadrivet ledarskap eller Ledarskapets ekonomi` (7,5 hp); rad: - Datadrivet ledarskap eller Ledarskapets ekonomi, 7,5 hp</t>
+          <t>`Logik och matematik` (7,5hp); rad: - Logik och matematik, 7,5hp</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DBIMA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DDCMA</t>
+          <t>DITMG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,24 +509,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bullet beskriver val mellan flera kurser</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>`Datadrivet ledarskap eller Ledarskapets ekonomi` (7,5 hp); rad: - Datadrivet ledarskap eller Ledarskapets ekonomi, 7,5 hp</t>
+          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5hp</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DDCMA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DITMG</t>
+          <t>DSVPG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`Logik och matematik` (7,5hp); rad: - Logik och matematik, 7,5hp</t>
+          <t>`Datakommunikation I` (7,5 hp); rad: - Datakommunikation I, 7,5 hp</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>DITMG</t>
+          <t>DSVPG</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5hp</t>
+          <t>`Data Storage &amp; Management Technologies` (7,5 hp); rad: - Data Storage &amp; Management Technologies, 7,5 hp</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>`Datakommunikation I` (7,5 hp); rad: - Datakommunikation I, 7,5 hp</t>
+          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5 hp</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -617,12 +617,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>`Data Storage &amp; Management Technologies` (7,5 hp); rad: - Data Storage &amp; Management Technologies, 7,5 hp</t>
+          <t>Programtext `Webbaserade geografiska informationssystem` ≠ kursplanens namn `Webbaserade geografiska informationssystem (GIS)` (kurskod `GIK2JX`); rad: - [[GIK2JX|Webbaserade geografiska informationssystem]], 7,5 hp</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DSVPG</t>
+          <t>KGDWG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -654,14 +654,14 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DSVPG</t>
+          <t>TATPG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -671,24 +671,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Programtext `Webbaserade geografiska informationssystem` ≠ kursplanens namn `Webbaserade geografiska informationssystem (GIS)` (kurskod `GIK2JX`); rad: - [[GIK2JX|Webbaserade geografiska informationssystem]], 7,5 hp</t>
+          <t>`Forskningsmetodik för ingenjörer` (7,5hp); rad: - Forskningsmetodik för ingenjörer, 7,5hp</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KGDWG</t>
+          <t>TATPG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -698,17 +698,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5 hp</t>
+          <t>`Examensarbete i assisterande teknik med inriktning mot maskinteknik` (15 hp); rad: - Examensarbete i assisterande teknik med inriktning mot maskinteknik, 15 hp</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`Forskningsmetodik för ingenjörer` (7,5hp); rad: - Forskningsmetodik för ingenjörer, 7,5hp</t>
+          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -742,7 +742,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TATPG</t>
+          <t>TBTCG</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -752,24 +752,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>`Examensarbete i assisterande teknik med inriktning mot maskinteknik` (15 hp); rad: - Examensarbete i assisterande teknik med inriktning mot maskinteknik, 15 hp</t>
+          <t>Programtext `Husbyggnadsprojekt I – Små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – Små byggnader och bostadsområden]], 15 hp</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TATPG</t>
+          <t>TBTCG</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -779,24 +779,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp</t>
+          <t>Programtext `Husbyggnadsprojekt III – Byggkonstruktionsprojekt` ≠ kursplanens namn `Husbyggnadsprojekt III - Byggkonstruktionsprojekt` (kurskod `GBY3AX`); rad: - [[GBY3AX|Husbyggnadsprojekt III – Byggkonstruktionsprojekt]], 7,5 hp</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TBTCG</t>
+          <t>TBTFG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt I – Små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – Små byggnader och bostadsområden]], 15 hp</t>
+          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTFG</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TBTCG</t>
+          <t>TBYSG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,24 +833,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt III – Byggkonstruktionsprojekt` ≠ kursplanens namn `Husbyggnadsprojekt III - Byggkonstruktionsprojekt` (kurskod `GBY3AX`); rad: - [[GBY3AX|Husbyggnadsprojekt III – Byggkonstruktionsprojekt]], 7,5 hp</t>
+          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TBTFG</t>
+          <t>TBYSG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -870,14 +870,14 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTFG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TBYSG</t>
+          <t>TEKHG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
+          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TBYSG</t>
+          <t>TEKHG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
+          <t>Programtext `Industriell ekonomi – organisation och ledarskap` ≠ kursplanens namn `Industriell ekonomi - organisation och ledarskap` (kurskod `GIE26M`); rad: - [[GIE26M|Industriell ekonomi – organisation och ledarskap]], 7,5 hp</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
+          <t>Programtext `Industriell ekonomi – underhåll och kvalitet` ≠ kursplanens namn `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`); rad: - [[GIE26N|Industriell ekonomi – underhåll och kvalitet]], 7,5 hp</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TEKHG</t>
+          <t>THIHG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -973,19 +973,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – organisation och ledarskap` ≠ kursplanens namn `Industriell ekonomi - organisation och ledarskap` (kurskod `GIE26M`); rad: - [[GIE26M|Industriell ekonomi – organisation och ledarskap]], 7,5 hp</t>
+          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TEKHG</t>
+          <t>THIHG</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1000,19 +1000,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – underhåll och kvalitet` ≠ kursplanens namn `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`); rad: - [[GIE26N|Industriell ekonomi – underhåll och kvalitet]], 7,5 hp</t>
+          <t>Programtext `Utvecklingsprojekt, tillverkning av en solfångare` ≠ kursplanens namn `Utvecklingsprojekt, tillverkning av en solfångare` (kurskod `GEG2JP`); rad: - [[GEG2JP|Utvecklingsprojekt, tillverkning av en solfångare]], 7,5 hp</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>THIHG</t>
+          <t>TMIEA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1027,19 +1027,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
+          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>THIHG</t>
+          <t>TMSSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1049,24 +1049,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursraden ser avbruten/feltrycklig ut</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Programtext `Utvecklingsprojekt, tillverkning av en solfångare` ≠ kursplanens namn `Utvecklingsprojekt, tillverkning av en solfångare` (kurskod `GEG2JP`); rad: - [[GEG2JP|Utvecklingsprojekt, tillverkning av en solfångare]], 7,5 hp</t>
+          <t>`Solenergiteknikpraktik (7,5 eller` (15 hp); rad: - Solenergiteknikpraktik (7,5 eller, 15 hp</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TMIEA</t>
+          <t>TMSSA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
+          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
         </is>
       </c>
     </row>
@@ -1103,12 +1103,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>`Solenergiteknikpraktik (7,5 eller` (15 hp); rad: - Solenergiteknikpraktik (7,5 eller, 15 hp</t>
+          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
+          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TMSSA</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1157,24 +1157,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
+          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TMSSA</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1184,24 +1184,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
+          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TPOKG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1216,12 +1216,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
+          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
+          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1292,12 +1292,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
+          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1309,7 +1309,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TSETA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1324,71 +1324,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
+          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Bullet beskriver val mellan flera kurser</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>`CAM / CNC` (7,5 hp); rad: - CAM / CNC, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>TSETA</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E35"/>
+  <autoFilter ref="A1:E33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1454,10 +1400,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course analysis files and exclude bullet points in program descriptions
- Added a new bullet point exclusion for "Solenergiteknikpraktik (7,5 eller" in checks_nedlagda.py.
- Updated various Excel files across multiple university departments (IIT, IHV, IKS, ISLL) to reflect changes in grading reports, grading scales, examination forms, phrasing consistency, knowledge requirements, introductory phrases, and references for discontinued courses.
- Corrected links and counts in markdown files related to program courses, ensuring accurate representation of linked and unlinked courses.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>`Solenergiteknikpraktik (7,5 eller` (15 hp); rad: - Solenergiteknikpraktik (7,5 eller, 15 hp</t>
+          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
+          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
+          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1120,7 +1120,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TMSSA</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
+          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TPOKG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
+          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
+          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
+          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
+          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1282,7 +1282,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TSETA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1292,49 +1292,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
+          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TSETA</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E33"/>
+  <autoFilter ref="A1:E32"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1398,8 +1371,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add normalization function for course name comparison and update related checks
- Introduced `_normalize_for_display_compare` function to standardize course name comparisons by collapsing whitespace, converting to lowercase, and preserving dash/slash variants.
- Updated `check_programtext_skiljer_kursnamn` to utilize the new normalization function for comparing displayed course names against canonical names.
- Adjusted documentation to reflect changes in whitespace handling and normalization process.
- Updated various Excel files and markdown documents to reflect changes in course name discrepancies and download links.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -985,7 +985,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>THIHG</t>
+          <t>TMIEA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1000,19 +1000,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Programtext `Utvecklingsprojekt, tillverkning av en solfångare` ≠ kursplanens namn `Utvecklingsprojekt, tillverkning av en solfångare` (kurskod `GEG2JP`); rad: - [[GEG2JP|Utvecklingsprojekt, tillverkning av en solfångare]], 7,5 hp</t>
+          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TMIEA</t>
+          <t>TMSSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
+          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
+          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
+          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TMSSA</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1103,24 +1103,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
+          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TPOKG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1135,12 +1135,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
+          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
+          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
+          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1238,12 +1238,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
+          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TSETA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1265,49 +1265,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
+          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TSETA</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E32"/>
+  <autoFilter ref="A1:E31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1369,8 +1342,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis Excel files with recent changes
- Modified "Programkurser olänkade.xlsx" to reflect updated data.
- Revised "Samstämighet svenska och engelska.xlsx" for consistency improvements.
- Corrected errors in "Stavfel och språkbruk.xlsx" to enhance accuracy.
- Updated "Övrigt.xlsx" with additional relevant information.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -487,7 +487,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`Logik och matematik` (7,5hp); rad: - Logik och matematik, 7,5hp</t>
+          <t>`Logik och matematik` (7,5hp); rad: - Logik och matematik, 7,5hp — sannolikt avses `Logik och matematik för datavetenskap` (kurskod `GMI23G`)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`Datakommunikation I` (7,5 hp); rad: - Datakommunikation I, 7,5 hp</t>
+          <t>`Datakommunikation I` (7,5 hp); rad: - Datakommunikation I, 7,5 hp — sannolikt avses `Datakommunikation 1` (kurskod `GDT2JM`)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`Data Storage &amp; Management Technologies` (7,5 hp); rad: - Data Storage &amp; Management Technologies, 7,5 hp</t>
+          <t>`Data Storage &amp; Management Technologies` (7,5 hp); rad: - Data Storage &amp; Management Technologies, 7,5 hp — sannolikt avses `Data Storage and Management Technologies` (kurskod `GIK2NV`)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp</t>
+          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp — sannolikt avses `Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -742,7 +742,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TBTCG</t>
+          <t>TBYSG</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -752,24 +752,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt I – Små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – Små byggnader och bostadsområden]], 15 hp</t>
+          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TBTCG</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -779,24 +779,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt III – Byggkonstruktionsprojekt` ≠ kursplanens namn `Husbyggnadsprojekt III - Byggkonstruktionsprojekt` (kurskod `GBY3AX`); rad: - [[GBY3AX|Husbyggnadsprojekt III – Byggkonstruktionsprojekt]], 7,5 hp</t>
+          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp — sannolikt avses `Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TBTFG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -806,24 +806,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
+          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp — sannolikt avses `3D-CAD – grundkurs` (kurskod `GMT338`)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTFG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TBYSG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -838,19 +838,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
+          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TBYSG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -860,24 +860,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp — sannolikt avses `Examensarbete för högskoleexamen i maskinteknik` (kurskod `GMT34W`)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TEKHG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
+          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp — sannolikt avses `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TEKHG</t>
+          <t>TPTAG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – organisation och ledarskap` ≠ kursplanens namn `Industriell ekonomi - organisation och ledarskap` (kurskod `GIE26M`); rad: - [[GIE26M|Industriell ekonomi – organisation och ledarskap]], 7,5 hp</t>
+          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TEKHG</t>
+          <t>TSETA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -941,346 +941,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Programtext `Industriell ekonomi – underhåll och kvalitet` ≠ kursplanens namn `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`); rad: - [[GIE26N|Industriell ekonomi – underhåll och kvalitet]], 7,5 hp</t>
+          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp — sannolikt avses `Design av PV- och hybridsystem` (kurskod `AEG26X`)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>THIHG</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>TMIEA</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TMSSA</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>TMSSA</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>TMSSA</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>TPOKG</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TPTAG</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Programtext avviker från kursplanens namn</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`); rad: - [[GMT34P|CAM / CNC]], 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>TSETA</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E31"/>
+  <autoFilter ref="A1:E19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1318,30 +994,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis files across multiple programs
- Modified various Excel files related to grading reporting, grading scales, Bloom's taxonomy, examination forms, and consistency in phrasing for the following programs: IIT, IHV, IKS, and ISLL.
- Updated markdown files for program courses and their references, ensuring accuracy in course names and descriptions.
- Adjusted binary files for consistency in naming and content across different program analyses.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp)</t>
+          <t>`Additiv tillverkning` (7,5 hp) — sannolikt avses `Additiv tillverkning (3D printing)` (kurskod `GMT34A`)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">

</xml_diff>

<commit_message>
Update analysis files across multiple departments with various corrections and improvements
- Updated Betygsrapportering.xlsx, Betygsskalor.xlsx, Bloom-taxonomi.xlsx, Examinationsformer.xlsx, Frasningskonsistens.xlsx, Förkunskapskrav.xlsx, Introfras.xlsx, Nedlagda kursreferenser.xlsx, Omfång på lärandemål.xlsx, Programkurser olänkade.xlsx, Samstämmighet svenska och engelska.xlsx, Stavfel och språkbruk.xlsx, and Övrigt.xlsx in the 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Adjusted content for accuracy and consistency across all documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -698,12 +698,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp)</t>
+          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp) — sannolikt avses `Fysisk planering III - genomförande och juridisk fördjupning` (kurskod `GSQ2PH`)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update course references and descriptions in educational plans
- Revised descriptions for unlinked program courses to clarify discrepancies between course names and curriculum titles across multiple educational plans.
- Updated binary files related to course analysis, reflecting changes in course data.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,6 +478,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Förslag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Länk</t>
         </is>
       </c>
@@ -509,10 +515,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>`Logik och matematik` (7,5hp) — sannolikt avses `Logik och matematik för datavetenskap` (kurskod `GMI23G`)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+          <t>`Logik och matematik` (7,5hp)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>`Logik och matematik för datavetenskap` (kurskod `GMI23G`)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
         </is>
@@ -546,10 +557,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+          <t>`System- och verksamhetsutveckling`</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>`System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
         </is>
@@ -579,10 +595,15 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`Datakommunikation I` (7,5 hp) — sannolikt avses `Datakommunikation 1` (kurskod `GDT2JM`)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+          <t>`Datakommunikation I` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>`Datakommunikation 1` (kurskod `GDT2JM`)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
@@ -612,10 +633,15 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`Data Storage &amp; Management Technologies` (7,5 hp) — sannolikt avses `Data Storage and Management Technologies` (kurskod `GIK2NV`)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+          <t>`Data Storage &amp; Management Technologies` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>`Data Storage and Management Technologies` (kurskod `GIK2NV`)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
@@ -645,10 +671,15 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+          <t>`System- och verksamhetsutveckling`</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>`System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
@@ -678,10 +709,15 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Programtext `Webbaserade geografiska informationssystem` ≠ kursplanens namn `Webbaserade geografiska informationssystem (GIS)` (kurskod `GIK2JX`)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+          <t>`Webbaserade geografiska informationssystem`</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>`Webbaserade geografiska informationssystem (GIS)` (kurskod `GIK2JX`)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
@@ -711,10 +747,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+          <t>`System- och verksamhetsutveckling`</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>`System och verksamhetsutveckling` (kurskod `GIK2XZ`)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
         </is>
@@ -744,10 +785,15 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden i praktiken` (7,5 hp) — sannolikt avses `Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+          <t>`Finita elementmetoden i praktiken` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>`Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
         </is>
@@ -781,10 +827,15 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp) — sannolikt avses `Fysisk planering III - genomförande och juridisk fördjupning` (kurskod `GSQ2PH`)</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
+          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>`Fysisk planering III - genomförande och juridisk fördjupning` (kurskod `GSQ2PH`)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
@@ -818,10 +869,15 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden` (7,5hp) — sannolikt avses `Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
+          <t>`Finita elementmetoden` (7,5hp)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>`Finita element metoden i praktiken` (kurskod `GMT2QF`)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
@@ -851,10 +907,15 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>`3D CAD grundkurs` (7,5 hp) — sannolikt avses `3D-CAD – grundkurs` (kurskod `GMT338`)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
+          <t>`3D CAD grundkurs` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>`3D-CAD – grundkurs` (kurskod `GMT338`)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
@@ -884,10 +945,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp) — sannolikt avses `Additiv tillverkning (3D printing)` (kurskod `GMT34A`)</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+          <t>`Additiv tillverkning` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>`Additiv tillverkning (3D printing)` (kurskod `GMT34A`)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
@@ -917,10 +983,15 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp) — sannolikt avses `Examensarbete för högskoleexamen i maskinteknik` (kurskod `GMT34W`)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>`Examensarbete för högskoleexamen i maskinteknik` (kurskod `GMT34W`)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
@@ -950,10 +1021,15 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>`Underhåll och kvalitet` (7,5 hp) — sannolikt avses `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
+          <t>`Underhåll och kvalitet` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>`Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
@@ -983,10 +1059,15 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Programtext `CAM / CNC` ≠ kursplanens namn `CAM/CNC` (kurskod `GMT34P`)</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
+          <t>`CAM / CNC`</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>`CAM/CNC` (kurskod `GMT34P`)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
         </is>
@@ -1020,50 +1101,55 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>`Design av PV hybrid system` (7,5 hp) — sannolikt avses `Design av PV- och hybridsystem` (kurskod `AEG26X`)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
+          <t>`Design av PV hybrid system` (7,5 hp)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>`Design av PV- och hybridsystem` (kurskod `AEG26X`)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:H17"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis and reports for Dalarna University programs
- Modified various Excel files related to grading reporting, grading scales, Bloom's taxonomy, examination forms, and consistency in phrasing across multiple programs (IIT, IHV, IKS, ISLL).
- Updated markdown files for program references, correcting discrepancies in course names and codes.
- Ensured all changes reflect the latest curriculum updates and maintain consistency in documentation across all departments.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olänkade.xlsx
@@ -590,17 +590,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Kurs finns aktivt men scrapern länkade inte</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`Datakommunikation I` (7,5 hp)</t>
+          <t>`Data Storage &amp; Management Technologies` (7,5 hp)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>`Datakommunikation 1` (kurskod `GDT2JM`)</t>
+          <t>`Data Storage and Management Technologies` (kurskod `GIK2NV`)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`Data Storage &amp; Management Technologies` (7,5 hp)</t>
+          <t>`Datakommunikation I`</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>`Data Storage and Management Technologies` (kurskod `GIK2NV`)</t>
+          <t>`Datakommunikation 1` (kurskod `GDT2JM`)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">

</xml_diff>